<commit_message>
test: align QA matrix with V6 contract
</commit_message>
<xml_diff>
--- a/plan-pruebas/matriz-pruebas/matriz-casos.xlsx
+++ b/plan-pruebas/matriz-pruebas/matriz-casos.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>director@blenkir.edu.pe / mbappe29</t>
+          <t>director@blenkir.edu.pe / DEMO_PASSWORD</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -959,17 +959,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>JSON 660+23 cuentas</t>
+          <t>JSON con las cuentas vigentes (usuario + rol), sin hashes ni contraseñas</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>accounts-export.controller</t>
+          <t>sin reejecución en la auditoría V6; la cifra histórica de la población demo no aplica</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1021,17 +1021,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Nuevo accessToken</t>
+          <t>200 + accessToken nuevo; logout invalida el refresh (401)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>pendiente ejecución dedicada</t>
+          <t>200 y refresh revocado · 39/39 integration tests (BD aislada, 2026-09-26)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Observado</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>backend/src/controllers/auth.controller.ts</t>
+          <t>evidencias-finales/terminal/integration-refactor-2026-20260926.log</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Menú admin 14 secciones</t>
+          <t>Menú admin 20 secciones</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>14 secciones</t>
+          <t>20 secciones</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>page.tsx L54-70</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>pruebas-caja-blanca/evidencias/auditoria-caja-blanca.json</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Menú docente 10 secciones</t>
+          <t>Menú docente 15 secciones</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10 secciones</t>
+          <t>15 secciones</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>page.tsx L71-82</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>evidencias-finales/capturas/dashboard-profesor-ok.png</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Menú estudiante 6 secciones</t>
+          <t>Menú estudiante 12 secciones</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1517,12 +1517,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6 secciones</t>
+          <t>12 secciones</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>page.tsx L83-90</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>evidencias-finales/capturas/dashboard-alumno-ok.png</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1822,17 +1822,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>52 modelos</t>
+          <t>57 modelos (54 activos + 3 legacy con @@ignore)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>modelos definidos</t>
+          <t>modelos contados por script</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>backend/prisma/schema.prisma</t>
+          <t>npm run db:count-models → 57 (2026-09-26)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>backend/prisma/schema.prisma</t>
+          <t>backend/scripts/count-prisma-models.mjs</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1879,22 +1879,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>npm run db:seed</t>
+          <t>npm run db:seed (db:seed:structure)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>seed.ts</t>
+          <t>prisma/seed.ts</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Grados, niveles</t>
+          <t>Grados, niveles y catálogos</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>db:seed OK</t>
+          <t>db:seed → tsx prisma/seed.ts</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1936,27 +1936,27 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>660 estudiantes demo</t>
+          <t>Población legacy deshabilitada</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>db:seed:demo</t>
+          <t>npm run db:seed:demo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>demo data</t>
+          <t>scripts/legacy-population-disabled.mjs</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>count=660</t>
+          <t>rechazo explícito sin escribir en la BD</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>seed demo</t>
+          <t>Error LEGACY + exit 1 (2026-09-26), BD intacta</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>backend/scripts/check-db.mjs</t>
+          <t>backend/scripts/legacy-population-disabled.mjs</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -1998,32 +1998,32 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>23 profesores</t>
+          <t>Listado docente</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>query teacher</t>
+          <t>GET /teachers</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>activos</t>
+          <t>admin token</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>count=23</t>
+          <t>lista paginada de profesores activos</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>profesores demo</t>
+          <t>captura histórica de la población demo anterior; revalidar en BD vigente</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2060,27 +2060,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bimestres III-IV vacíos</t>
+          <t>Períodos académicos 2026</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>validate-demo-data</t>
+          <t>resolvePeriodoByParam</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>periodo 3-4</t>
+          <t>BD aislada de pruebas</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0 notas</t>
+          <t>periodo III 2026 activo y evidencia restringida al año 2026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>seed-grades.ts</t>
+          <t>39/39 integration tests (2026-09-26)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>backend/prisma/seed-grades.ts</t>
+          <t>evidencias-finales/terminal/integration-refactor-2026-20260926.log</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2137,17 +2137,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>201 matriculaId</t>
+          <t>201 + matriculaId</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>pendiente POST dedicado</t>
+          <t>201 item.id=15 persistida en BD aislada (2026-09-26)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Observado</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>backend/src/routes/index.ts</t>
+          <t>evidencias-finales/api/matricula-post-201-aislado-20260926.json</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2184,27 +2184,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Entrenar ensemble</t>
+          <t>Artefactos del modelo V6</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>npm run ml:train</t>
+          <t>artifacts/synthetic/</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>train.py</t>
+          <t>entrenamiento 2026-09-24</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>best_model.joblib</t>
+          <t>best_model.joblib + metadata.json + metrics.json</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>models/ generados</t>
+          <t>model_version BLENKIR_V6_BIN_20260924</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>machine-learning/models/metrics.json</t>
+          <t>machine-learning/artifacts/synthetic/metadata.json</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>pytest predict</t>
+          <t>Suite de pruebas ML</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>6+ tests pass</t>
+          <t>32 tests pass</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>pruebas-unitarias/evidencias/ml-tests.log</t>
+          <t>32/32 (2026-09-26)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2308,27 +2308,27 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Heurística riesgo bajo</t>
+          <t>Nivel bajo por umbral</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>promedio 16 asist 95</t>
+          <t>probabilidad 0.40</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>payload bajo</t>
+          <t>payload válido</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>level=bajo</t>
+          <t>level=bajo (p &lt; 0.41)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>test_heuristic_low_risk</t>
+          <t>test_probability_to_level_matches_thresholds</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2370,27 +2370,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Heurística riesgo alto</t>
+          <t>Nivel alto por umbral</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>promedio 8 retirado</t>
+          <t>probabilidad 0.70</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>payload alto</t>
+          <t>payload válido</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>level medio|alto</t>
+          <t>level=alto (p &gt;= 0.65)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>test_heuristic_high_risk</t>
+          <t>test_high_probability_maps_to_alto</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vector 10 features</t>
+          <t>Vector de 7 features</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>shape (1,10)</t>
+          <t>shape (1,7) y orden del contrato</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>app/features.py</t>
+          <t>test_exactly_seven_features + test_features_shape_and_order</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DELETE attendance admin</t>
+          <t>DELETE reportes solo admin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>DELETE /attendance/:id docente</t>
+          <t>DELETE /reports/:id token docente</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3129,17 +3129,17 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>403 Permiso denegado</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>routes L206</t>
+          <t>authorize(admin) en routes/index.ts; sin ejecución automatizada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4059,17 +4059,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>660 estudiantes KPI</t>
+          <t>kpis.byLevel, riskTrend y modelComparison</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>dashboard-director-ok.png</t>
+          <t>captura histórica de la población demo anterior</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Listado 23 docentes</t>
+          <t>Listado docente</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4183,17 +4183,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>23 filas</t>
+          <t>tabla paginada con buscador por nombre, código, especialidad o correo</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>HTTP 200 count≈0 (67ms)</t>
+          <t>captura previa al refresh V6; reejecución pendiente</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>evidencias-finales/api/teachers-list.json</t>
+          <t>evidencias-finales/capturas/profesores-listado.png</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>14 módulos director</t>
+          <t>20 secciones director</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5366,12 +5366,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>capturas director</t>
+          <t>UAT histórico ejecutado con 14 secciones; reejecución pendiente tras el refresh V6</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">

</xml_diff>

<commit_message>
chore: close BLENKIR V6 technical audit
Squash merge PR #6: align BLENKIR V6 documentation, QA/ISO evidence, frontend branding, ML V6 references, GitHub metadata and repository consistency. Sonar code fixes remain for a separate follow-up PR.
</commit_message>
<xml_diff>
--- a/plan-pruebas/matriz-pruebas/matriz-casos.xlsx
+++ b/plan-pruebas/matriz-pruebas/matriz-casos.xlsx
@@ -582,7 +582,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>director@blenkir.edu.pe / mbappe29</t>
+          <t>director@blenkir.edu.pe / DEMO_PASSWORD</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -959,17 +959,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>JSON 660+23 cuentas</t>
+          <t>JSON con las cuentas vigentes (usuario + rol), sin hashes ni contraseñas</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>accounts-export.controller</t>
+          <t>sin reejecución en la auditoría V6; la cifra histórica de la población demo no aplica</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1021,17 +1021,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Nuevo accessToken</t>
+          <t>200 + accessToken nuevo; logout invalida el refresh (401)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>pendiente ejecución dedicada</t>
+          <t>200 y refresh revocado · 39/39 integration tests (BD aislada, 2026-09-26)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Observado</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>backend/src/controllers/auth.controller.ts</t>
+          <t>evidencias-finales/terminal/integration-refactor-2026-20260926.log</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Menú admin 14 secciones</t>
+          <t>Menú admin 20 secciones</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>14 secciones</t>
+          <t>20 secciones</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>page.tsx L54-70</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>pruebas-caja-blanca/evidencias/auditoria-caja-blanca.json</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Menú docente 10 secciones</t>
+          <t>Menú docente 15 secciones</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10 secciones</t>
+          <t>15 secciones</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>page.tsx L71-82</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>evidencias-finales/capturas/dashboard-profesor-ok.png</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Menú estudiante 6 secciones</t>
+          <t>Menú estudiante 12 secciones</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1517,12 +1517,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6 secciones</t>
+          <t>12 secciones</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>page.tsx L83-90</t>
+          <t>role-sections.test.ts PASS</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>evidencias-finales/capturas/dashboard-alumno-ok.png</t>
+          <t>frontend/tests/role-sections.test.ts</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1822,17 +1822,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>52 modelos</t>
+          <t>57 modelos (54 activos + 3 legacy con @@ignore)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>modelos definidos</t>
+          <t>modelos contados por script</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>backend/prisma/schema.prisma</t>
+          <t>npm run db:count-models → 57 (2026-09-26)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>backend/prisma/schema.prisma</t>
+          <t>backend/scripts/count-prisma-models.mjs</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1879,22 +1879,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>npm run db:seed</t>
+          <t>npm run db:seed (db:seed:structure)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>seed.ts</t>
+          <t>prisma/seed.ts</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Grados, niveles</t>
+          <t>Grados, niveles y catálogos</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>db:seed OK</t>
+          <t>db:seed → tsx prisma/seed.ts</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1936,27 +1936,27 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>660 estudiantes demo</t>
+          <t>Población legacy deshabilitada</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>db:seed:demo</t>
+          <t>npm run db:seed:demo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>demo data</t>
+          <t>scripts/legacy-population-disabled.mjs</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>count=660</t>
+          <t>rechazo explícito sin escribir en la BD</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>seed demo</t>
+          <t>Error LEGACY + exit 1 (2026-09-26), BD intacta</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>backend/scripts/check-db.mjs</t>
+          <t>backend/scripts/legacy-population-disabled.mjs</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -1998,32 +1998,32 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>23 profesores</t>
+          <t>Listado docente</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>query teacher</t>
+          <t>GET /teachers</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>activos</t>
+          <t>admin token</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>count=23</t>
+          <t>lista paginada de profesores activos</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>profesores demo</t>
+          <t>captura histórica de la población demo anterior; revalidar en BD vigente</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2060,27 +2060,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bimestres III-IV vacíos</t>
+          <t>Períodos académicos 2026</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>validate-demo-data</t>
+          <t>resolvePeriodoByParam</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>periodo 3-4</t>
+          <t>BD aislada de pruebas</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0 notas</t>
+          <t>periodo III 2026 activo y evidencia restringida al año 2026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>seed-grades.ts</t>
+          <t>39/39 integration tests (2026-09-26)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>backend/prisma/seed-grades.ts</t>
+          <t>evidencias-finales/terminal/integration-refactor-2026-20260926.log</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2137,17 +2137,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>201 matriculaId</t>
+          <t>201 + matriculaId</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>pendiente POST dedicado</t>
+          <t>201 item.id=15 persistida en BD aislada (2026-09-26)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Observado</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>backend/src/routes/index.ts</t>
+          <t>evidencias-finales/api/matricula-post-201-aislado-20260926.json</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2184,27 +2184,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Entrenar ensemble</t>
+          <t>Artefactos del modelo V6</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>npm run ml:train</t>
+          <t>artifacts/synthetic/</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>train.py</t>
+          <t>entrenamiento 2026-09-24</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>best_model.joblib</t>
+          <t>best_model.joblib + metadata.json + metrics.json</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>models/ generados</t>
+          <t>model_version BLENKIR_V6_BIN_20260924</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>machine-learning/models/metrics.json</t>
+          <t>machine-learning/artifacts/synthetic/metadata.json</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>pytest predict</t>
+          <t>Suite de pruebas ML</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2261,12 +2261,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>6+ tests pass</t>
+          <t>32 tests pass</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>pruebas-unitarias/evidencias/ml-tests.log</t>
+          <t>32/32 (2026-09-26)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2308,27 +2308,27 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Heurística riesgo bajo</t>
+          <t>Nivel bajo por umbral</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>promedio 16 asist 95</t>
+          <t>probabilidad 0.40</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>payload bajo</t>
+          <t>payload válido</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>level=bajo</t>
+          <t>level=bajo (p &lt; 0.41)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>test_heuristic_low_risk</t>
+          <t>test_probability_to_level_matches_thresholds</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2370,27 +2370,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Heurística riesgo alto</t>
+          <t>Nivel alto por umbral</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>promedio 8 retirado</t>
+          <t>probabilidad 0.70</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>payload alto</t>
+          <t>payload válido</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>level medio|alto</t>
+          <t>level=alto (p &gt;= 0.65)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>test_heuristic_high_risk</t>
+          <t>test_high_probability_maps_to_alto</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vector 10 features</t>
+          <t>Vector de 7 features</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>shape (1,10)</t>
+          <t>shape (1,7) y orden del contrato</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>app/features.py</t>
+          <t>test_exactly_seven_features + test_features_shape_and_order</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DELETE attendance admin</t>
+          <t>DELETE reportes solo admin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>DELETE /attendance/:id docente</t>
+          <t>DELETE /reports/:id token docente</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3129,17 +3129,17 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>403 Permiso denegado</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>routes L206</t>
+          <t>authorize(admin) en routes/index.ts; sin ejecución automatizada</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4059,17 +4059,17 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>660 estudiantes KPI</t>
+          <t>kpis.byLevel, riskTrend y modelComparison</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>dashboard-director-ok.png</t>
+          <t>captura histórica de la población demo anterior</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4168,7 +4168,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Listado 23 docentes</t>
+          <t>Listado docente</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4183,17 +4183,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>23 filas</t>
+          <t>tabla paginada con buscador por nombre, código, especialidad o correo</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>HTTP 200 count≈0 (67ms)</t>
+          <t>captura previa al refresh V6; reejecución pendiente</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>evidencias-finales/api/teachers-list.json</t>
+          <t>evidencias-finales/capturas/profesores-listado.png</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>14 módulos director</t>
+          <t>20 secciones director</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5366,12 +5366,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>capturas director</t>
+          <t>UAT histórico ejecutado con 14 secciones; reejecución pendiente tras el refresh V6</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Aprobado</t>
+          <t>Observado</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">

</xml_diff>